<commit_message>
auto: session 2026-10-27 11:15
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/11-bao-gia-khach/Bao-Gia-PR-Thanh-Nien-Trung-Tam-Piano-2026-10-27.xlsx
+++ b/11-bao-gia-khach/Bao-Gia-PR-Thanh-Nien-Trung-Tam-Piano-2026-10-27.xlsx
@@ -645,11 +645,11 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>01 bài PR tối đa 1.000 chữ, 5 ảnh, 2 hyperlink. Tiêu đề tối đa 17 chữ, sapo 60 chữ. Duyệt bài khoảng 3-5 ngày làm việc (không tính thứ Bảy, Chủ nhật).</t>
+          <t>01 bài PR tối đa 1.000 chữ, 5 ảnh, 2 hyperlink, đăng tại tiểu mục phù hợp với nội dung bài.</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>17820000</v>
+        <v>15010000</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
@@ -657,10 +657,10 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>13365000</v>
+        <v>11255000</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>14434200</v>
+        <v>12155400</v>
       </c>
     </row>
     <row r="11" ht="64" customHeight="1">
@@ -1013,9 +1013,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>